<commit_message>
Fix overview export filenames (ref/exp column fallback).
Co-authored-by: frankrita0728-coder <frankrita0728-coder@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/pairing_results/2609-21_ZE1_list/analysis_results.xlsx
+++ b/data/pairing_results/2609-21_ZE1_list/analysis_results.xlsx
@@ -535,6 +535,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_a09_1.csv</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>09-09_11-19-17_426_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I2" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -610,6 +620,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_a09_2.csv</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>09-09_11-21-27_792_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I3" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -685,6 +705,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_a10_1.csv</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>09-09_11-23-48_013_ExgCh1Data_(Frank 右脛前肌)_a10_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -760,6 +790,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_a10_2.csv</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>09-09_11-25-35_742_ExgCh1Data_(Frank 右脛前肌)_a10_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -835,6 +875,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_ze2_1.csv</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>09-09_11-27-57_319_Ch2_(Frank 右脛前肌)_ze2_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I6" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -910,6 +960,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2609-09 frank右脛前肌(Delsys)_with_ze2_2.csv</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>09-09_11-30-01_689_Ch2_(Frank 右脛前肌)_ze2_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -985,6 +1045,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_a09_1.csv</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>09-09_09-41-19_786_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1060,6 +1130,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_a09_2.csv</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>09-09_09-45-46_944_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I9" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1135,6 +1215,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_a10_1.csv</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>09-09_09-52-57_312_ExgCh2Data_(Frank 左脛前肌)_a10_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I10" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1210,6 +1300,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_a10_2.csv</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>09-09_09-58-36_663_ExgCh2Data_(Frank 左脛前肌)_a10_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I11" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1285,6 +1385,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_ze2_1.csv</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>09-09_10-8-56_879_Ch1_(Frank_左脛前肌)_ze2_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I12" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1360,6 +1470,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2609-09 frank左脛前肌(Delsys)_with_ze2_2.csv</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>09-09_10-12-46_289_Ch1_(Frank 左脛前肌)_ze2_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I13" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1435,6 +1555,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2609-09 frank右腓腸肌(Delsys)_with_a09_1.csv</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>09-09_11-48-01_319_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1508,6 +1638,12 @@
       <c r="F15" t="inlineStr">
         <is>
           <t>3</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>09-09_11-50-05_808_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_2.txt</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1565,6 +1701,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2609-09 frank右腓腸肌(Delsys)_with_a10_1.csv</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>09-09_11-52-29_385_ExgCh2Data_(Frank 右腓腸肌)_a10_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I16" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1640,6 +1786,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2609-09 frank右腓腸肌(Delsys)_with_a10_2.csv</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>09-09_11-55-52_064_ExgCh2Data_(Frank 右腓腸肌)_a10_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1715,6 +1871,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2609-09 frank右腓腸肌(Delsys)_with_ZE2_1.csv</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>09-09_11-59-10_048_Ch1_(Frank 右腓腸肌)_ze2_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1790,6 +1956,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2609-09 frank右腓腸肌(Delsys)_with_ZE2_2.csv</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>09-09_12-1-14_084_Ch1_(Frank 右腓腸肌)_ze2_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1865,6 +2041,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_a09_1.csv</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>09-09_10-31-15_181_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -1940,6 +2126,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_a09_2.csv</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>09-09_10-35-51_625_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I21" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2015,6 +2211,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_a10_1.csv</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>09-09_10-40-13_031_ExgCh1Data_(Frank 左腓腸肌)_a10_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2090,6 +2296,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_a10_2.csv</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>09-09_10-45-37_881_ExgCh1Data_(Frank 左腓腸肌)_a10_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I23" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2165,6 +2381,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_ze2_1.csv</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>09-09_10-48-41_826_Ch2_(Frank 左腓腸肌)_ze2_褲XL_1.txt</t>
+        </is>
+      </c>
       <c r="I24" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2240,6 +2466,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2609-09 frank左腓腸肌(Delsys)_with_ze2_2.csv</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>09-09_10-51-00_016_Ch2_(Frank 左腓腸肌)_ze2_褲XL_2.txt</t>
+        </is>
+      </c>
       <c r="I25" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2315,6 +2551,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>09-09_11-19-17_426_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>09-09_14-55-41_279_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_去腿毛.txt</t>
+        </is>
+      </c>
       <c r="I26" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2390,6 +2636,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>09-09_09-41-19_786_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>09-09_12-39-13_023_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_去腿毛.txt</t>
+        </is>
+      </c>
       <c r="I27" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2465,6 +2721,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>09-09_11-48-01_319_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>09-09_15-16-55_610_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_去腿毛.txt</t>
+        </is>
+      </c>
       <c r="I28" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2540,6 +2806,16 @@
           <t>3</t>
         </is>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>09-09_10-31-15_181_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_1.txt</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>09-09_14-32-12_387_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_去腿毛.txt</t>
+        </is>
+      </c>
       <c r="I29" t="inlineStr">
         <is>
           <t>3/3</t>
@@ -2615,6 +2891,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右脛前肌_a09_褲XL_疲勞1.csv</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>09-09_14-57-46_856_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_疲勞1.txt</t>
+        </is>
+      </c>
       <c r="I30" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -2690,6 +2976,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右脛前肌_a09_褲XL_疲勞2.csv</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>09-09_15-01-03_995_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_疲勞2.txt</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -2765,6 +3061,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右脛前肌_a09_褲XL_疲勞3.csv</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>09-09_15-05-27_867_ExgCh1Data_(Frank 右脛前肌)_a09_褲XL_疲勞3.txt</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -2840,6 +3146,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左脛前肌_a09_褲XL_疲勞1.csv</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>09-09_12-42-56_134_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_疲勞1.txt</t>
+        </is>
+      </c>
       <c r="I33" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -2915,6 +3231,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左脛前肌_a09_褲XL_疲勞2.csv</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>09-09_12-47-55_198_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_疲勞2.txt</t>
+        </is>
+      </c>
       <c r="I34" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -2990,6 +3316,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左脛前肌_a09_褲XL_疲勞3.csv</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>09-09_12-51-53_172_ExgCh2Data_(Frank 左脛前肌)_a09_褲XL_疲勞3.txt</t>
+        </is>
+      </c>
       <c r="I35" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3065,6 +3401,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右腓腸肌_a09_褲XL_疲勞1.csv</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>09-09_15-20-08_195_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_疲勞1.txt</t>
+        </is>
+      </c>
       <c r="I36" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3140,6 +3486,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右腓腸肌_a09_褲XL_疲勞2.csv</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>09-09_15-23-04_934_ExgCh2Data_(Frank 右腓腸肌)_a09_褲XL_疲勞2.txt</t>
+        </is>
+      </c>
       <c r="I37" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3215,6 +3571,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2609-09 frank 右腓腸肌_a09_褲XL_疲勞3.csv</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>09-09_15-25-56_272_ExgCh2Data(Frank 右腓腸肌)_a09_褲XL_疲勞3.txt</t>
+        </is>
+      </c>
       <c r="I38" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3290,6 +3656,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左腓腸肌_a09_褲XL_疲勞1.csv</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>09-09_14-34-47_174_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_疲勞1.txt</t>
+        </is>
+      </c>
       <c r="I39" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3365,6 +3741,16 @@
           <t>10</t>
         </is>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左腓腸肌_a09_褲XL_疲勞2.csv</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>09-09_14-38-43_403_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_疲勞2.txt</t>
+        </is>
+      </c>
       <c r="I40" t="inlineStr">
         <is>
           <t>10/10</t>
@@ -3438,6 +3824,16 @@
       <c r="F41" t="inlineStr">
         <is>
           <t>10</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2609-09 frank 左腓腸肌_a09_褲XL_疲勞3.csv</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>09-09_14-42-34_881_ExgCh1Data_(Frank 左腓腸肌)_a09_褲XL_疲勞3.txt</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">

</xml_diff>